<commit_message>
#8 Transmitter BOM Button Changed Main Board PCB routing in progress
</commit_message>
<xml_diff>
--- a/Design-Files/Transmitter433MHz-v1.0/Deliverables/BOM/Client BOM.xlsx
+++ b/Design-Files/Transmitter433MHz-v1.0/Deliverables/BOM/Client BOM.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\hasanmehmood-motordriver\Design-Files\Transmitter433MHz-v1.0\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -51,9 +51,6 @@
     <t>Battery Connector</t>
   </si>
   <si>
-    <t>Metal Dome Pot</t>
-  </si>
-  <si>
     <t>Inductor</t>
   </si>
   <si>
@@ -93,9 +90,6 @@
     <t>J1</t>
   </si>
   <si>
-    <t>J3, J4, J5, J6</t>
-  </si>
-  <si>
     <t>L1</t>
   </si>
   <si>
@@ -156,9 +150,6 @@
     <t>Battery button CR2032 Plugin Battery Connectors ROHS</t>
   </si>
   <si>
-    <t>Circular 160gf 0.25mm - Metal Dome Pot ROHS</t>
-  </si>
-  <si>
     <t>FIXED IND 180NH 150MA 3.38OHM SM</t>
   </si>
   <si>
@@ -207,9 +198,6 @@
     <t>MY-2032-02</t>
   </si>
   <si>
-    <t>600-508S-160</t>
-  </si>
-  <si>
     <t>IND-0402</t>
   </si>
   <si>
@@ -297,9 +285,6 @@
     <t>MYOUNG</t>
   </si>
   <si>
-    <t>HYP</t>
-  </si>
-  <si>
     <t>FH</t>
   </si>
   <si>
@@ -394,6 +379,21 @@
   </si>
   <si>
     <t>Panasonic</t>
+  </si>
+  <si>
+    <t>Switch</t>
+  </si>
+  <si>
+    <t>SW1, SW2, SW3, SW4</t>
+  </si>
+  <si>
+    <t>SWITCH TACTILE SPST-NO 0.05A 12V</t>
+  </si>
+  <si>
+    <t>B3U-1000P</t>
+  </si>
+  <si>
+    <t>Omron</t>
   </si>
 </sst>
 </file>
@@ -905,6 +905,9 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -913,9 +916,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1282,9 +1282,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
+      <c r="I1" s="56"/>
+      <c r="J1" s="56"/>
+      <c r="K1" s="56"/>
     </row>
     <row r="2" spans="1:11" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="51" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="3"/>
@@ -1312,13 +1312,13 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="52" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
-      <c r="K3" s="56"/>
+      <c r="K3" s="57"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1329,13 +1329,13 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="53" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="6"/>
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
-      <c r="K4" s="57"/>
+      <c r="K4" s="58"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1352,7 +1352,7 @@
       <c r="H5" s="5"/>
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
-      <c r="K5" s="57"/>
+      <c r="K5" s="58"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1365,7 +1365,7 @@
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
-      <c r="K6" s="57"/>
+      <c r="K6" s="58"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1378,7 +1378,7 @@
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
-      <c r="K7" s="57"/>
+      <c r="K7" s="58"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1391,7 +1391,7 @@
       <c r="H8" s="7"/>
       <c r="I8" s="7"/>
       <c r="J8" s="7"/>
-      <c r="K8" s="57"/>
+      <c r="K8" s="58"/>
     </row>
     <row r="9" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1402,28 +1402,28 @@
         <v>6</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="J9" s="29" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="K9" s="29" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1432,26 +1432,26 @@
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="58" t="s">
+      <c r="C10" s="55" t="s">
         <v>7</v>
       </c>
       <c r="D10" s="36" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F10" s="36" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G10" s="37" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="I10" s="37" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="J10" s="36">
         <v>1</v>
@@ -1464,26 +1464,26 @@
         <f t="shared" ref="B11:B30" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="58" t="s">
+      <c r="C11" s="55" t="s">
         <v>8</v>
       </c>
       <c r="D11" s="38" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E11" s="39" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G11" s="39" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="I11" s="39" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="J11" s="38">
         <v>2</v>
@@ -1496,26 +1496,26 @@
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="58" t="s">
+      <c r="C12" s="55" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="36" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F12" s="36" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G12" s="37" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="H12" s="36" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="I12" s="37" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="J12" s="36">
         <v>1</v>
@@ -1528,26 +1528,26 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="58" t="s">
+      <c r="C13" s="55" t="s">
         <v>8</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E13" s="39" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F13" s="38" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G13" s="39" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="H13" s="38" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="I13" s="39" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="J13" s="38">
         <v>1</v>
@@ -1560,26 +1560,26 @@
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="58" t="s">
+      <c r="C14" s="55" t="s">
         <v>8</v>
       </c>
       <c r="D14" s="36" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E14" s="37" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F14" s="36" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G14" s="37" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H14" s="36" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="I14" s="37" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="J14" s="36">
         <v>1</v>
@@ -1592,26 +1592,26 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="58" t="s">
+      <c r="C15" s="55" t="s">
         <v>8</v>
       </c>
       <c r="D15" s="38" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E15" s="39" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G15" s="39" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="H15" s="38" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="I15" s="39" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="J15" s="38">
         <v>1</v>
@@ -1624,319 +1624,319 @@
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="58" t="s">
+      <c r="C16" s="55" t="s">
         <v>9</v>
       </c>
       <c r="D16" s="36" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="F16" s="36" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G16" s="37" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="H16" s="36" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="I16" s="37" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="J16" s="36">
         <v>1</v>
       </c>
       <c r="K16" s="36"/>
     </row>
-    <row r="17" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B17) - ROW($B$9)</f>
         <v>8</v>
       </c>
-      <c r="C17" s="58" t="s">
+      <c r="C17" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="D17" s="38" t="s">
-        <v>24</v>
-      </c>
-      <c r="E17" s="39" t="s">
-        <v>45</v>
-      </c>
-      <c r="F17" s="38" t="s">
-        <v>62</v>
-      </c>
-      <c r="G17" s="39" t="s">
-        <v>62</v>
-      </c>
-      <c r="H17" s="38" t="s">
-        <v>92</v>
-      </c>
-      <c r="I17" s="39" t="s">
-        <v>62</v>
-      </c>
-      <c r="J17" s="38">
-        <v>4</v>
-      </c>
-      <c r="K17" s="38"/>
-    </row>
-    <row r="18" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D17" s="36" t="s">
+        <v>23</v>
+      </c>
+      <c r="E17" s="37" t="s">
+        <v>43</v>
+      </c>
+      <c r="F17" s="36" t="s">
+        <v>59</v>
+      </c>
+      <c r="G17" s="37" t="s">
+        <v>71</v>
+      </c>
+      <c r="H17" s="36" t="s">
+        <v>85</v>
+      </c>
+      <c r="I17" s="37" t="s">
+        <v>101</v>
+      </c>
+      <c r="J17" s="36">
+        <v>1</v>
+      </c>
+      <c r="K17" s="36"/>
+    </row>
+    <row r="18" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="50">
-        <f>ROW(B18) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="58" t="s">
-        <v>11</v>
-      </c>
-      <c r="D18" s="36" t="s">
-        <v>25</v>
-      </c>
-      <c r="E18" s="37" t="s">
-        <v>46</v>
-      </c>
-      <c r="F18" s="36" t="s">
-        <v>63</v>
-      </c>
-      <c r="G18" s="37" t="s">
-        <v>75</v>
-      </c>
-      <c r="H18" s="36" t="s">
-        <v>89</v>
-      </c>
-      <c r="I18" s="37" t="s">
-        <v>106</v>
-      </c>
-      <c r="J18" s="36">
+      <c r="C18" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="38" t="s">
+        <v>24</v>
+      </c>
+      <c r="E18" s="39" t="s">
+        <v>44</v>
+      </c>
+      <c r="F18" s="38" t="s">
+        <v>59</v>
+      </c>
+      <c r="G18" s="39" t="s">
+        <v>72</v>
+      </c>
+      <c r="H18" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="I18" s="39" t="s">
+        <v>102</v>
+      </c>
+      <c r="J18" s="38">
         <v>1</v>
       </c>
-      <c r="K18" s="36"/>
+      <c r="K18" s="38"/>
     </row>
     <row r="19" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B19) - ROW($B$9)</f>
         <v>10</v>
       </c>
-      <c r="C19" s="58" t="s">
-        <v>11</v>
-      </c>
-      <c r="D19" s="38" t="s">
-        <v>26</v>
-      </c>
-      <c r="E19" s="39" t="s">
-        <v>47</v>
-      </c>
-      <c r="F19" s="38" t="s">
-        <v>63</v>
-      </c>
-      <c r="G19" s="39" t="s">
-        <v>76</v>
-      </c>
-      <c r="H19" s="38" t="s">
-        <v>93</v>
-      </c>
-      <c r="I19" s="39" t="s">
-        <v>107</v>
-      </c>
-      <c r="J19" s="38">
+      <c r="C19" s="55" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="36" t="s">
+        <v>25</v>
+      </c>
+      <c r="E19" s="37" t="s">
+        <v>45</v>
+      </c>
+      <c r="F19" s="36" t="s">
+        <v>59</v>
+      </c>
+      <c r="G19" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="H19" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="I19" s="37" t="s">
+        <v>103</v>
+      </c>
+      <c r="J19" s="36">
         <v>1</v>
       </c>
-      <c r="K19" s="38"/>
+      <c r="K19" s="36"/>
     </row>
     <row r="20" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="50">
-        <f>ROW(B20) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="58" t="s">
+      <c r="C20" s="55" t="s">
         <v>11</v>
       </c>
-      <c r="D20" s="36" t="s">
-        <v>27</v>
-      </c>
-      <c r="E20" s="37" t="s">
-        <v>48</v>
-      </c>
-      <c r="F20" s="36" t="s">
-        <v>63</v>
-      </c>
-      <c r="G20" s="37" t="s">
-        <v>77</v>
-      </c>
-      <c r="H20" s="36" t="s">
-        <v>94</v>
-      </c>
-      <c r="I20" s="37" t="s">
-        <v>108</v>
-      </c>
-      <c r="J20" s="36">
+      <c r="D20" s="38" t="s">
+        <v>26</v>
+      </c>
+      <c r="E20" s="39" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="38" t="s">
+        <v>60</v>
+      </c>
+      <c r="G20" s="39" t="s">
+        <v>74</v>
+      </c>
+      <c r="H20" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="I20" s="39" t="s">
+        <v>104</v>
+      </c>
+      <c r="J20" s="38">
         <v>1</v>
       </c>
-      <c r="K20" s="36"/>
-    </row>
-    <row r="21" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K20" s="38"/>
+    </row>
+    <row r="21" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B21) - ROW($B$9)</f>
         <v>12</v>
       </c>
-      <c r="C21" s="58" t="s">
+      <c r="C21" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="D21" s="38" t="s">
-        <v>28</v>
-      </c>
-      <c r="E21" s="39" t="s">
-        <v>49</v>
-      </c>
-      <c r="F21" s="38" t="s">
-        <v>64</v>
-      </c>
-      <c r="G21" s="39" t="s">
-        <v>78</v>
-      </c>
-      <c r="H21" s="38" t="s">
-        <v>95</v>
-      </c>
-      <c r="I21" s="39" t="s">
-        <v>109</v>
-      </c>
-      <c r="J21" s="38">
-        <v>1</v>
-      </c>
-      <c r="K21" s="38"/>
-    </row>
-    <row r="22" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D21" s="36" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>47</v>
+      </c>
+      <c r="F21" s="36" t="s">
+        <v>61</v>
+      </c>
+      <c r="G21" s="37" t="s">
+        <v>75</v>
+      </c>
+      <c r="H21" s="36" t="s">
+        <v>86</v>
+      </c>
+      <c r="I21" s="37" t="s">
+        <v>105</v>
+      </c>
+      <c r="J21" s="36">
+        <v>2</v>
+      </c>
+      <c r="K21" s="36"/>
+    </row>
+    <row r="22" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="50">
-        <f>ROW(B22) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="58" t="s">
-        <v>13</v>
-      </c>
-      <c r="D22" s="36" t="s">
-        <v>29</v>
-      </c>
-      <c r="E22" s="37" t="s">
-        <v>50</v>
-      </c>
-      <c r="F22" s="36" t="s">
-        <v>65</v>
-      </c>
-      <c r="G22" s="37" t="s">
-        <v>79</v>
-      </c>
-      <c r="H22" s="36" t="s">
-        <v>90</v>
-      </c>
-      <c r="I22" s="37" t="s">
-        <v>110</v>
-      </c>
-      <c r="J22" s="36">
-        <v>2</v>
-      </c>
-      <c r="K22" s="36"/>
+      <c r="C22" s="55" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="38" t="s">
+        <v>28</v>
+      </c>
+      <c r="E22" s="39" t="s">
+        <v>48</v>
+      </c>
+      <c r="F22" s="38" t="s">
+        <v>61</v>
+      </c>
+      <c r="G22" s="39" t="s">
+        <v>76</v>
+      </c>
+      <c r="H22" s="38" t="s">
+        <v>91</v>
+      </c>
+      <c r="I22" s="39" t="s">
+        <v>106</v>
+      </c>
+      <c r="J22" s="38">
+        <v>1</v>
+      </c>
+      <c r="K22" s="38"/>
     </row>
     <row r="23" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B23) - ROW($B$9)</f>
         <v>14</v>
       </c>
-      <c r="C23" s="58" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" s="38" t="s">
-        <v>30</v>
-      </c>
-      <c r="E23" s="39" t="s">
-        <v>51</v>
-      </c>
-      <c r="F23" s="38" t="s">
-        <v>65</v>
-      </c>
-      <c r="G23" s="39" t="s">
-        <v>80</v>
-      </c>
-      <c r="H23" s="38" t="s">
-        <v>96</v>
-      </c>
-      <c r="I23" s="39" t="s">
-        <v>111</v>
-      </c>
-      <c r="J23" s="38">
+      <c r="C23" s="55" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="36" t="s">
+        <v>29</v>
+      </c>
+      <c r="E23" s="37" t="s">
+        <v>49</v>
+      </c>
+      <c r="F23" s="36" t="s">
+        <v>61</v>
+      </c>
+      <c r="G23" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="H23" s="36" t="s">
+        <v>91</v>
+      </c>
+      <c r="I23" s="37" t="s">
+        <v>107</v>
+      </c>
+      <c r="J23" s="36">
         <v>1</v>
       </c>
-      <c r="K23" s="38"/>
+      <c r="K23" s="36"/>
     </row>
     <row r="24" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="50">
-        <f>ROW(B24) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="58" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24" s="36" t="s">
-        <v>31</v>
-      </c>
-      <c r="E24" s="37" t="s">
-        <v>52</v>
-      </c>
-      <c r="F24" s="36" t="s">
-        <v>65</v>
-      </c>
-      <c r="G24" s="37" t="s">
-        <v>81</v>
-      </c>
-      <c r="H24" s="36" t="s">
-        <v>96</v>
-      </c>
-      <c r="I24" s="37" t="s">
-        <v>112</v>
-      </c>
-      <c r="J24" s="36">
+      <c r="C24" s="55" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="38" t="s">
+        <v>30</v>
+      </c>
+      <c r="E24" s="39" t="s">
+        <v>50</v>
+      </c>
+      <c r="F24" s="38" t="s">
+        <v>61</v>
+      </c>
+      <c r="G24" s="39" t="s">
+        <v>78</v>
+      </c>
+      <c r="H24" s="38" t="s">
+        <v>86</v>
+      </c>
+      <c r="I24" s="39" t="s">
+        <v>108</v>
+      </c>
+      <c r="J24" s="38">
         <v>1</v>
       </c>
-      <c r="K24" s="36"/>
+      <c r="K24" s="38"/>
     </row>
     <row r="25" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="50">
-        <f t="shared" si="0"/>
+        <f>ROW(B25) - ROW($B$9)</f>
         <v>16</v>
       </c>
-      <c r="C25" s="58" t="s">
-        <v>13</v>
-      </c>
-      <c r="D25" s="38" t="s">
-        <v>32</v>
-      </c>
-      <c r="E25" s="39" t="s">
-        <v>53</v>
-      </c>
-      <c r="F25" s="38" t="s">
-        <v>65</v>
-      </c>
-      <c r="G25" s="39" t="s">
-        <v>82</v>
-      </c>
-      <c r="H25" s="38" t="s">
-        <v>90</v>
-      </c>
-      <c r="I25" s="39" t="s">
-        <v>113</v>
-      </c>
-      <c r="J25" s="38">
+      <c r="C25" s="55" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="36" t="s">
+        <v>31</v>
+      </c>
+      <c r="E25" s="37" t="s">
+        <v>51</v>
+      </c>
+      <c r="F25" s="36" t="s">
+        <v>61</v>
+      </c>
+      <c r="G25" s="37" t="s">
+        <v>79</v>
+      </c>
+      <c r="H25" s="36" t="s">
+        <v>86</v>
+      </c>
+      <c r="I25" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="J25" s="36">
         <v>1</v>
       </c>
-      <c r="K25" s="38"/>
+      <c r="K25" s="36"/>
     </row>
     <row r="26" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
@@ -1944,29 +1944,29 @@
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
       </c>
-      <c r="C26" s="58" t="s">
-        <v>13</v>
+      <c r="C26" s="55" t="s">
+        <v>120</v>
       </c>
       <c r="D26" s="36" t="s">
-        <v>33</v>
+        <v>121</v>
       </c>
       <c r="E26" s="37" t="s">
-        <v>54</v>
+        <v>122</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>65</v>
+        <v>123</v>
       </c>
       <c r="G26" s="37" t="s">
-        <v>83</v>
+        <v>123</v>
       </c>
       <c r="H26" s="36" t="s">
-        <v>90</v>
+        <v>124</v>
       </c>
       <c r="I26" s="37" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="J26" s="36">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K26" s="36"/>
     </row>
@@ -1976,26 +1976,26 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C27" s="58" t="s">
-        <v>14</v>
+      <c r="C27" s="55" t="s">
+        <v>13</v>
       </c>
       <c r="D27" s="38" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E27" s="39" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="F27" s="38" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="G27" s="39" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="H27" s="38" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="I27" s="39" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="J27" s="38">
         <v>1</v>
@@ -2008,26 +2008,26 @@
         <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
-      <c r="C28" s="58" t="s">
-        <v>14</v>
+      <c r="C28" s="55" t="s">
+        <v>13</v>
       </c>
       <c r="D28" s="36" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E28" s="37" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G28" s="37" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="H28" s="36" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="I28" s="37" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="J28" s="36">
         <v>1</v>
@@ -2040,26 +2040,26 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C29" s="58" t="s">
-        <v>15</v>
+      <c r="C29" s="55" t="s">
+        <v>14</v>
       </c>
       <c r="D29" s="38" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E29" s="39" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F29" s="38" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G29" s="39" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="H29" s="38" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="I29" s="39" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="J29" s="38">
         <v>1</v>
@@ -2072,26 +2072,26 @@
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C30" s="58" t="s">
-        <v>120</v>
+      <c r="C30" s="55" t="s">
+        <v>115</v>
       </c>
       <c r="D30" s="38" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="E30" s="38" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="F30" s="38" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="G30" s="38" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="H30" s="38" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="I30" s="38" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="J30" s="38">
         <v>1</v>

</xml_diff>